<commit_message>
add reset to subdisplay
</commit_message>
<xml_diff>
--- a/pcb/bill_of_materials.xlsx
+++ b/pcb/bill_of_materials.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="150">
   <si>
     <t>No.</t>
   </si>
@@ -205,7 +205,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C28,C29,C30,C31</t>
+    <t>C28,C29,C30,C31,C32</t>
   </si>
   <si>
     <t>MBK0805X7R104K500NT</t>
@@ -220,6 +220,42 @@
     <t>13</t>
   </si>
   <si>
+    <t>330nF</t>
+  </si>
+  <si>
+    <t>C33</t>
+  </si>
+  <si>
+    <t>CAP-SMD_L3.2-W1.6</t>
+  </si>
+  <si>
+    <t>CA45A-A-35V-0.33UF-K</t>
+  </si>
+  <si>
+    <t>CEC(振华新云)</t>
+  </si>
+  <si>
+    <t>C2976917</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>C34</t>
+  </si>
+  <si>
+    <t>CAP-SMD_L3.2-W1.6-RD</t>
+  </si>
+  <si>
+    <t>CA45-A-35V-0.1UF-K</t>
+  </si>
+  <si>
+    <t>C2976900</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
     <t>SS12</t>
   </si>
   <si>
@@ -232,7 +268,7 @@
     <t>C379819</t>
   </si>
   <si>
-    <t>14</t>
+    <t>16</t>
   </si>
   <si>
     <t>AFA07-S09FCC-00</t>
@@ -250,7 +286,7 @@
     <t>C262343</t>
   </si>
   <si>
-    <t>15</t>
+    <t>17</t>
   </si>
   <si>
     <t>B-2100S15P-A110</t>
@@ -268,7 +304,7 @@
     <t>C124373</t>
   </si>
   <si>
-    <t>16</t>
+    <t>18</t>
   </si>
   <si>
     <t>IL-AG5-10P-S3L2</t>
@@ -286,7 +322,7 @@
     <t>C2891425</t>
   </si>
   <si>
-    <t>17</t>
+    <t>19</t>
   </si>
   <si>
     <t>470nH</t>
@@ -307,7 +343,7 @@
     <t>C295221</t>
   </si>
   <si>
-    <t>18</t>
+    <t>20</t>
   </si>
   <si>
     <t>CD4066BM</t>
@@ -325,7 +361,7 @@
     <t>C353979</t>
   </si>
   <si>
-    <t>19</t>
+    <t>21</t>
   </si>
   <si>
     <t>XL2515</t>
@@ -343,7 +379,7 @@
     <t>C609744</t>
   </si>
   <si>
-    <t>20</t>
+    <t>22</t>
   </si>
   <si>
     <t>9.1k</t>
@@ -355,7 +391,7 @@
     <t>R0805</t>
   </si>
   <si>
-    <t>21</t>
+    <t>23</t>
   </si>
   <si>
     <t>2.4k</t>
@@ -364,7 +400,7 @@
     <t>R21</t>
   </si>
   <si>
-    <t>22</t>
+    <t>24</t>
   </si>
   <si>
     <t>10k</t>
@@ -373,54 +409,24 @@
     <t>R23</t>
   </si>
   <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>1kΩ</t>
-  </si>
-  <si>
-    <t>R24,R25</t>
-  </si>
-  <si>
-    <t>RMC08051K1%N</t>
+    <t>25</t>
+  </si>
+  <si>
+    <t>220Ω</t>
+  </si>
+  <si>
+    <t>R28,R29,R30,R32</t>
+  </si>
+  <si>
+    <t>R1206</t>
+  </si>
+  <si>
+    <t>RMC12062205%N</t>
   </si>
   <si>
     <t>Tyohm(幸亚电阻)</t>
   </si>
   <si>
-    <t>C269744</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>2kΩ</t>
-  </si>
-  <si>
-    <t>R26,R27</t>
-  </si>
-  <si>
-    <t>RMC08052K1%N</t>
-  </si>
-  <si>
-    <t>C269745</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>220Ω</t>
-  </si>
-  <si>
-    <t>R28,R29,R30</t>
-  </si>
-  <si>
-    <t>R1206</t>
-  </si>
-  <si>
-    <t>RMC12062205%N</t>
-  </si>
-  <si>
     <t>C269757</t>
   </si>
   <si>
@@ -437,6 +443,24 @@
   </si>
   <si>
     <t>C269751</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>78L09</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>SOT-89-3_L4.5-W2.5-P1.50-LS4.2-BR</t>
+  </si>
+  <si>
+    <t>DOWO(东沃)</t>
+  </si>
+  <si>
+    <t>C6718416</t>
   </si>
 </sst>
 </file>
@@ -813,7 +837,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="11" width="20" customWidth="1"/>
@@ -1244,7 +1268,7 @@
         <v>62</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" t="s">
         <v>63</v>
@@ -1291,16 +1315,16 @@
         <v>71</v>
       </c>
       <c r="F14" t="s">
-        <v>15</v>
+        <v>69</v>
       </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H14" t="s">
-        <v>15</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J14" t="s">
         <v>19</v>
@@ -1311,63 +1335,63 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" t="s">
         <v>73</v>
       </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" t="s">
-        <v>75</v>
-      </c>
-      <c r="E15" t="s">
-        <v>76</v>
-      </c>
-      <c r="F15" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" t="s">
-        <v>74</v>
-      </c>
-      <c r="H15" t="s">
-        <v>77</v>
-      </c>
       <c r="I15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J15" t="s">
         <v>19</v>
       </c>
       <c r="K15" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
+        <v>82</v>
+      </c>
+      <c r="E16" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" t="s">
         <v>81</v>
       </c>
-      <c r="E16" t="s">
-        <v>82</v>
-      </c>
-      <c r="F16" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" t="s">
-        <v>80</v>
-      </c>
       <c r="H16" t="s">
-        <v>83</v>
+        <v>15</v>
       </c>
       <c r="I16" t="s">
         <v>84</v>
@@ -1376,7 +1400,7 @@
         <v>19</v>
       </c>
       <c r="K16" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1384,7 +1408,7 @@
         <v>85</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" t="s">
         <v>86</v>
@@ -1411,7 +1435,7 @@
         <v>19</v>
       </c>
       <c r="K17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1419,7 +1443,7 @@
         <v>91</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="s">
         <v>92</v>
@@ -1434,77 +1458,77 @@
         <v>15</v>
       </c>
       <c r="G18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H18" t="s">
         <v>95</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>96</v>
-      </c>
-      <c r="I18" t="s">
-        <v>97</v>
       </c>
       <c r="J18" t="s">
         <v>19</v>
       </c>
       <c r="K18" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
         <v>98</v>
       </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>99</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>100</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" t="s">
+        <v>98</v>
+      </c>
+      <c r="H19" t="s">
         <v>101</v>
       </c>
-      <c r="F19" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" t="s">
-        <v>99</v>
-      </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>102</v>
-      </c>
-      <c r="I19" t="s">
-        <v>103</v>
       </c>
       <c r="J19" t="s">
         <v>19</v>
       </c>
       <c r="K19" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
         <v>104</v>
       </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>105</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>106</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" t="s">
         <v>107</v>
-      </c>
-      <c r="F20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" t="s">
-        <v>105</v>
       </c>
       <c r="H20" t="s">
         <v>108</v>
@@ -1516,7 +1540,7 @@
         <v>19</v>
       </c>
       <c r="K20" t="s">
-        <v>98</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -1539,71 +1563,71 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>15</v>
+        <v>111</v>
       </c>
       <c r="H21" t="s">
-        <v>15</v>
+        <v>114</v>
       </c>
       <c r="I21" t="s">
-        <v>15</v>
+        <v>115</v>
       </c>
       <c r="J21" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K21" t="s">
-        <v>20</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F22" t="s">
         <v>15</v>
       </c>
       <c r="G22" t="s">
-        <v>15</v>
+        <v>117</v>
       </c>
       <c r="H22" t="s">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="I22" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="J22" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="K22" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D23" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E23" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="F23" t="s">
         <v>15</v>
@@ -1626,34 +1650,34 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D24" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E24" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="F24" t="s">
-        <v>121</v>
+        <v>15</v>
       </c>
       <c r="G24" t="s">
-        <v>123</v>
+        <v>15</v>
       </c>
       <c r="H24" t="s">
-        <v>124</v>
+        <v>15</v>
       </c>
       <c r="I24" t="s">
-        <v>125</v>
+        <v>15</v>
       </c>
       <c r="J24" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="K24" t="s">
         <v>20</v>
@@ -1661,34 +1685,34 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D25" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="F25" t="s">
-        <v>127</v>
+        <v>15</v>
       </c>
       <c r="G25" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="H25" t="s">
-        <v>124</v>
+        <v>15</v>
       </c>
       <c r="I25" t="s">
-        <v>130</v>
+        <v>15</v>
       </c>
       <c r="J25" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="K25" t="s">
         <v>20</v>
@@ -1696,31 +1720,31 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
+        <v>134</v>
+      </c>
+      <c r="E26" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" t="s">
         <v>133</v>
       </c>
-      <c r="E26" t="s">
-        <v>134</v>
-      </c>
-      <c r="F26" t="s">
-        <v>132</v>
-      </c>
       <c r="G26" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H26" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="I26" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="J26" t="s">
         <v>19</v>
@@ -1731,31 +1755,31 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>139</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
+        <v>140</v>
+      </c>
+      <c r="D27" t="s">
+        <v>141</v>
+      </c>
+      <c r="E27" t="s">
+        <v>135</v>
+      </c>
+      <c r="F27" t="s">
+        <v>140</v>
+      </c>
+      <c r="G27" t="s">
+        <v>142</v>
+      </c>
+      <c r="H27" t="s">
         <v>137</v>
       </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
-        <v>138</v>
-      </c>
-      <c r="D27" t="s">
-        <v>139</v>
-      </c>
-      <c r="E27" t="s">
-        <v>134</v>
-      </c>
-      <c r="F27" t="s">
-        <v>138</v>
-      </c>
-      <c r="G27" t="s">
-        <v>140</v>
-      </c>
-      <c r="H27" t="s">
-        <v>124</v>
-      </c>
       <c r="I27" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J27" t="s">
         <v>19</v>
@@ -1764,8 +1788,43 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>144</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
+        <v>145</v>
+      </c>
+      <c r="D28" t="s">
+        <v>146</v>
+      </c>
+      <c r="E28" t="s">
+        <v>147</v>
+      </c>
+      <c r="F28" t="s">
+        <v>15</v>
+      </c>
+      <c r="G28" t="s">
+        <v>145</v>
+      </c>
+      <c r="H28" t="s">
+        <v>148</v>
+      </c>
+      <c r="I28" t="s">
+        <v>149</v>
+      </c>
+      <c r="J28" t="s">
+        <v>19</v>
+      </c>
+      <c r="K28" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>